<commit_message>
edited a few files
</commit_message>
<xml_diff>
--- a/Session 5 - Chain Table/Answers/DS Lab report sheet.xlsx
+++ b/Session 5 - Chain Table/Answers/DS Lab report sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Files\DS_ChainTable\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\varin\Documents\Data Structure Git\Data-Structure-Library-1402\Session 5 - Chain Table\Answers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA34398D-161B-4D39-817F-BABF87DBB643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33331A01-9AFA-4A57-896E-B4903A9C7A3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t xml:space="preserve">Student Name </t>
   </si>
@@ -62,12 +62,6 @@
   </si>
   <si>
     <t>(time scale, ms/sec/...)</t>
-  </si>
-  <si>
-    <t>محمدرضا امینی</t>
-  </si>
-  <si>
-    <t>سید محمد مهدی رضوی</t>
   </si>
   <si>
     <t>Windows 11</t>
@@ -211,29 +205,29 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -456,10 +450,10 @@
   <dimension ref="A1:F18"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="25.109375" style="6" customWidth="1"/>
-    <col min="6" max="6" width="26.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="25.109375" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="12.6640625" style="6"/>
+    <col min="1" max="5" width="25.109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="25.109375" style="5" customWidth="1"/>
+    <col min="10" max="16384" width="12.6640625" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="13.2">
@@ -469,43 +463,35 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
     </row>
     <row r="2" spans="1:6" ht="48">
-      <c r="A2" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="7">
-        <v>402222020</v>
-      </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
+      <c r="A2" s="9"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
     </row>
     <row r="3" spans="1:6" ht="48">
-      <c r="A3" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="7">
-        <v>402222073</v>
-      </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
+      <c r="A3" s="9"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
     </row>
     <row r="4" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="7"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="6"/>
     </row>
     <row r="5" spans="1:6" ht="13.2">
       <c r="A5" s="3" t="s">
@@ -523,56 +509,56 @@
       <c r="E5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="7"/>
+      <c r="F5" s="6"/>
     </row>
     <row r="6" spans="1:6" ht="22.5" customHeight="1">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="12">
+      <c r="D6" s="10">
         <v>8</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="10">
         <v>4.5999999999999996</v>
       </c>
-      <c r="F6" s="7"/>
+      <c r="F6" s="6"/>
     </row>
     <row r="7" spans="1:6" ht="22.5" customHeight="1">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
     </row>
     <row r="8" spans="1:6" ht="26.25" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
+        <v>17</v>
+      </c>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
     </row>
     <row r="9" spans="1:6" ht="22.5" customHeight="1">
-      <c r="A9" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
+      <c r="A9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
     </row>
     <row r="10" spans="1:6" ht="26.25" customHeight="1">
-      <c r="A10" s="9"/>
+      <c r="A10" s="7"/>
     </row>
     <row r="11" spans="1:6" ht="26.25" customHeight="1">
       <c r="A11" s="4" t="s">
@@ -595,29 +581,29 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="22.5" customHeight="1">
-      <c r="A12" s="6">
+      <c r="A12" s="5">
         <v>10000</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="5">
         <v>6.0515732765197701</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="5">
         <v>9.9914073944091797E-3</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="5">
         <v>1.10034942626953E-2</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="5">
         <v>9.9914073944091797E-3</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>21</v>
+      <c r="F12" s="8" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="22.5" customHeight="1"/>
     <row r="14" spans="1:6" ht="22.5" customHeight="1">
-      <c r="F14" s="10" t="s">
-        <v>22</v>
+      <c r="F14" s="8" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="22.5" customHeight="1"/>

</xml_diff>